<commit_message>
create excel file data & use Data Provider for validate product creation
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AUTOMATION TEST\ProjectTest2025\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9580D9-188D-4190-A1FF-5C7572E45167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84475D0F-48E3-4E69-A6DA-EE783B5F9DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2820" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21450" yWindow="1020" windowWidth="20190" windowHeight="9390" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="d" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="bookLoginData" sheetId="5" r:id="rId3"/>
     <sheet name="emplVerification" sheetId="3" r:id="rId4"/>
     <sheet name="invalidLoginData" sheetId="2" r:id="rId5"/>
+    <sheet name="invalidProductData" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="35">
   <si>
     <t>username</t>
   </si>
@@ -65,13 +66,82 @@
   </si>
   <si>
     <t>abcde12345-</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>provider</t>
+  </si>
+  <si>
+    <t>productCode</t>
+  </si>
+  <si>
+    <t>productName</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>Item 1</t>
+  </si>
+  <si>
+    <t>KIM CHI</t>
+  </si>
+  <si>
+    <t>Sản phẩm 2</t>
+  </si>
+  <si>
+    <t>This is our best seller product</t>
+  </si>
+  <si>
+    <t>TH00</t>
+  </si>
+  <si>
+    <t>TcName</t>
+  </si>
+  <si>
+    <t>Blank Product Code</t>
+  </si>
+  <si>
+    <t>Blank all</t>
+  </si>
+  <si>
+    <t>Blank product Name</t>
+  </si>
+  <si>
+    <t>Blank unit</t>
+  </si>
+  <si>
+    <t>Blank description</t>
+  </si>
+  <si>
+    <t>Blank price</t>
+  </si>
+  <si>
+    <t>Blank quantity</t>
+  </si>
+  <si>
+    <t>Blank supplier</t>
+  </si>
+  <si>
+    <t>Blank category</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,6 +153,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -109,12 +187,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -568,4 +647,266 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C953E27E-A1BE-414F-8296-0BE51F7E32CB}">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2">
+        <v>30000</v>
+      </c>
+      <c r="I2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4">
+        <v>30000</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5">
+        <v>30000</v>
+      </c>
+      <c r="I5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>30000</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9">
+        <v>30000</v>
+      </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10">
+        <v>30000</v>
+      </c>
+      <c r="I10">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>